<commit_message>
schedule time update fromfrontend feature implemented
</commit_message>
<xml_diff>
--- a/data/connectivity.xlsx
+++ b/data/connectivity.xlsx
@@ -11,13 +11,14 @@
     <sheet sheetId="2" name="Connectivity 2026-10-03" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Connectivity 2026-10-04" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Connectivity 2026-10-05" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Connectivity 2026-10-07" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="195">
   <si>
     <t>IPSec Connectivity Check — 01 Oct 2026</t>
   </si>
@@ -607,6 +608,57 @@
   </si>
   <si>
     <t xml:space="preserve">          ESP spi in/out: 0xae4629e3/0xc12b43ea  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Active SA: 11</t>
+  </si>
+  <si>
+    <t>Total IKE SA: 11</t>
+  </si>
+  <si>
+    <t>1   IKE Peer: 180.211.232.98</t>
+  </si>
+  <si>
+    <t>2   IKE Peer: 220.247.161.226</t>
+  </si>
+  <si>
+    <t>3   IKE Peer: 119.30.37.30</t>
+  </si>
+  <si>
+    <t>4   IKE Peer: 103.230.107.231</t>
+  </si>
+  <si>
+    <t>5   IKE Peer: 203.223.93.33</t>
+  </si>
+  <si>
+    <t>6   IKE Peer: 103.134.91.14</t>
+  </si>
+  <si>
+    <t>7   IKE Peer: 119.40.82.243</t>
+  </si>
+  <si>
+    <t>9   IKE Peer: 182.163.98.81</t>
+  </si>
+  <si>
+    <t>11  IKE Peer: 202.84.44.65</t>
+  </si>
+  <si>
+    <t>Session-id:8701, Status:UP-ACTIVE, IKE count:1, CHILD count:3</t>
+  </si>
+  <si>
+    <t>1779345265 103.17.181.122/500                                  203.13.162.84/500                                        READY    INITIATOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Life/Active Time: 86400/611 sec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0xdf6e8334/0xc2aefe29  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0x4da2ab7f/0x7ba5603a  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0xd4bec43e/0xae7dc2dc  </t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -3263,7 +3315,7 @@
     </row>
     <row r="67" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E67" s="9" t="s">
-        <v>177</v>
+        <v>154</v>
       </c>
     </row>
     <row r="68" spans="5:5" x14ac:dyDescent="0.25">
@@ -3273,6 +3325,522 @@
     </row>
     <row r="69" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E69" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E60"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="3" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" t="s">
+        <v>96</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" t="s">
+        <v>96</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" t="s">
+        <v>96</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" t="s">
+        <v>96</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>127</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" t="s">
+        <v>96</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E24" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="9" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E26" s="9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E27" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E28" s="9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="9" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="32" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E32" s="9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E34" s="9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E35" s="9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E36" s="9" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E37" s="9" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E38" s="9" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E39" s="9" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E40" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E41" s="9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="42" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E43" s="9" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="44" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E44" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E45" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E46" s="9" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="9" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="48" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E48" s="9" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E49" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E50" s="9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E51" s="9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E52" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E53" s="9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E54" s="9" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E55" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E56" s="9" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E57" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E58" s="9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="59" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E59" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E60" s="9" t="s">
         <v>55</v>
       </c>
     </row>

</xml_diff>

<commit_message>
asa output as image and sheet fix
</commit_message>
<xml_diff>
--- a/data/connectivity.xlsx
+++ b/data/connectivity.xlsx
@@ -12,13 +12,15 @@
     <sheet sheetId="3" name="Connectivity 2026-10-04" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Connectivity 2026-10-05" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Connectivity 2026-10-07" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="07.10.2026" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="08.10.2026" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="215">
   <si>
     <t>IPSec Connectivity Check — 01 Oct 2026</t>
   </si>
@@ -659,6 +661,66 @@
   </si>
   <si>
     <t xml:space="preserve">          ESP spi in/out: 0xd4bec43e/0xae7dc2dc  </t>
+  </si>
+  <si>
+    <t>3   IKE Peer: 203.223.93.33</t>
+  </si>
+  <si>
+    <t>4   IKE Peer: 119.40.82.243</t>
+  </si>
+  <si>
+    <t>5   IKE Peer: 182.163.98.81</t>
+  </si>
+  <si>
+    <t>8   IKE Peer: 180.211.232.98</t>
+  </si>
+  <si>
+    <t>9   IKE Peer: 103.230.107.231</t>
+  </si>
+  <si>
+    <t>Session-id:41876, Status:UP-ACTIVE, IKE count:1, CHILD count:1</t>
+  </si>
+  <si>
+    <t>2220921289 103.17.181.122/4500                                 20.224.142.31/4500                                       READY    RESPONDER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Life/Active Time: 86400/1676 sec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0x4551c09f/0xc881e7b4  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Life/Active Time: 86400/35811 sec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0xe153fcd4/0x338e658b  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0xc4f4c029/0x143f1ad4  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0x7dae5095/0x60fb72f7  </t>
+  </si>
+  <si>
+    <t>2   IKE Peer: 119.40.82.243</t>
+  </si>
+  <si>
+    <t>4   IKE Peer: 192.144.80.90</t>
+  </si>
+  <si>
+    <t>7   IKE Peer: 103.230.107.231</t>
+  </si>
+  <si>
+    <t>Session-id:2210, Status:UP-ACTIVE, IKE count:1, CHILD count:1</t>
+  </si>
+  <si>
+    <t>467681251 103.17.181.122/4500                                 20.224.142.31/4500                                       READY    RESPONDER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Life/Active Time: 86400/60 sec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0x83ae90a2/0xc881ea37  </t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -738,7 +800,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -753,11 +815,26 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -780,6 +857,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3831,7 +3911,7 @@
     </row>
     <row r="58" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E58" s="9" t="s">
-        <v>194</v>
+        <v>154</v>
       </c>
     </row>
     <row r="59" spans="5:5" x14ac:dyDescent="0.25">
@@ -3841,6 +3921,948 @@
     </row>
     <row r="60" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E60" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E63"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="3" customWidth="1"/>
+    <col min="5" max="5" width="110" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E24" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="11" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E26" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E27" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E28" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E32" s="11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E34" s="11" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E35" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E36" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E37" s="11" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E38" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E39" s="11" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E40" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="41" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E41" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="42" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="43" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E43" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E44" s="11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="45" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E45" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E46" s="11" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E48" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E49" s="11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E50" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E51" s="11" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E52" s="11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E53" s="11" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E54" s="11" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E55" s="11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E56" s="11" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E57" s="11" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E58" s="11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="59" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E59" s="11" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="60" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E60" s="11" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="61" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E61" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="62" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E62" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E63" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="3" customWidth="1"/>
+    <col min="5" max="5" width="110" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E24" s="11" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E26" s="11" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E27" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E28" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="32" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E32" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="11" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E34" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E35" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E36" s="11" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E37" s="11" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E38" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E39" s="11" t="s">
         <v>55</v>
       </c>
     </row>

</xml_diff>

<commit_message>
qadmin and telegram issue fixed
</commit_message>
<xml_diff>
--- a/data/connectivity.xlsx
+++ b/data/connectivity.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="219">
   <si>
     <t>IPSec Connectivity Check — 01 Oct 2026</t>
   </si>
@@ -702,25 +702,37 @@
     <t xml:space="preserve">          ESP spi in/out: 0x7dae5095/0x60fb72f7  </t>
   </si>
   <si>
-    <t>2   IKE Peer: 119.40.82.243</t>
-  </si>
-  <si>
-    <t>4   IKE Peer: 192.144.80.90</t>
-  </si>
-  <si>
-    <t>7   IKE Peer: 103.230.107.231</t>
-  </si>
-  <si>
-    <t>Session-id:2210, Status:UP-ACTIVE, IKE count:1, CHILD count:1</t>
-  </si>
-  <si>
-    <t>467681251 103.17.181.122/4500                                 20.224.142.31/4500                                       READY    RESPONDER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      Life/Active Time: 86400/60 sec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">          ESP spi in/out: 0x83ae90a2/0xc881ea37  </t>
+    <t>3   IKE Peer: 103.230.107.231</t>
+  </si>
+  <si>
+    <t>4   IKE Peer: 180.211.232.98</t>
+  </si>
+  <si>
+    <t>5   IKE Peer: 119.30.37.30</t>
+  </si>
+  <si>
+    <t>6   IKE Peer: 119.40.82.243</t>
+  </si>
+  <si>
+    <t>7   IKE Peer: 203.223.93.33</t>
+  </si>
+  <si>
+    <t>9   IKE Peer: 103.134.91.14</t>
+  </si>
+  <si>
+    <t>11  IKE Peer: 82.149.6.229</t>
+  </si>
+  <si>
+    <t>Session-id:12323, Status:UP-ACTIVE, IKE count:1, CHILD count:1</t>
+  </si>
+  <si>
+    <t>3047503765 103.17.181.122/4500                                 20.224.142.31/4500                                       READY    RESPONDER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Life/Active Time: 86400/1058 sec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0x53e45326/0xc881eb7f  </t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -4463,7 +4475,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -4526,7 +4538,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>207</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -4568,7 +4580,7 @@
         <v>96</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -4582,7 +4594,7 @@
         <v>96</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -4624,7 +4636,7 @@
         <v>96</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -4652,7 +4664,7 @@
         <v>8</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -4694,7 +4706,7 @@
         <v>96</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>184</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -4708,7 +4720,7 @@
         <v>96</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -4736,7 +4748,7 @@
         <v>96</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -4750,7 +4762,7 @@
         <v>96</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -4778,12 +4790,12 @@
         <v>96</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>197</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E23" s="11" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="5:5" x14ac:dyDescent="0.25">
@@ -4792,63 +4804,63 @@
       </c>
     </row>
     <row r="25" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E25" s="9" t="s">
-        <v>8</v>
+      <c r="E25" s="11" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="26" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E26" s="11" t="s">
-        <v>137</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E27" s="9" t="s">
-        <v>8</v>
+      <c r="E27" s="11" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E28" s="11" t="s">
-        <v>210</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E29" s="9" t="s">
-        <v>8</v>
+      <c r="E29" s="11" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="30" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E30" s="11" t="s">
-        <v>139</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E31" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="32" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E32" s="11" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="33" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E33" s="11" t="s">
-        <v>212</v>
+        <v>136</v>
       </c>
     </row>
     <row r="34" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E34" s="11" t="s">
-        <v>143</v>
+      <c r="E34" s="9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E35" s="11" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="36" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E36" s="11" t="s">
-        <v>213</v>
+      <c r="E36" s="9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="37" spans="5:5" x14ac:dyDescent="0.25">
@@ -4863,6 +4875,51 @@
     </row>
     <row r="39" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E39" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E40" s="11" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E41" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="42" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="11" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="43" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E43" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="44" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E44" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="45" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E45" s="11" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E46" s="11" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E48" s="11" t="s">
         <v>55</v>
       </c>
     </row>

</xml_diff>

<commit_message>
tg diplicate issue fixed
</commit_message>
<xml_diff>
--- a/data/connectivity.xlsx
+++ b/data/connectivity.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="219">
   <si>
     <t>IPSec Connectivity Check — 01 Oct 2026</t>
   </si>
@@ -702,37 +702,37 @@
     <t xml:space="preserve">          ESP spi in/out: 0x7dae5095/0x60fb72f7  </t>
   </si>
   <si>
+    <t>2   IKE Peer: 103.134.91.14</t>
+  </si>
+  <si>
     <t>3   IKE Peer: 103.230.107.231</t>
   </si>
   <si>
     <t>4   IKE Peer: 180.211.232.98</t>
   </si>
   <si>
-    <t>5   IKE Peer: 119.30.37.30</t>
-  </si>
-  <si>
     <t>6   IKE Peer: 119.40.82.243</t>
   </si>
   <si>
-    <t>7   IKE Peer: 203.223.93.33</t>
-  </si>
-  <si>
-    <t>9   IKE Peer: 103.134.91.14</t>
-  </si>
-  <si>
-    <t>11  IKE Peer: 82.149.6.229</t>
-  </si>
-  <si>
-    <t>Session-id:12323, Status:UP-ACTIVE, IKE count:1, CHILD count:1</t>
-  </si>
-  <si>
-    <t>3047503765 103.17.181.122/4500                                 20.224.142.31/4500                                       READY    RESPONDER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      Life/Active Time: 86400/1058 sec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">          ESP spi in/out: 0x53e45326/0xc881eb7f  </t>
+    <t>7   IKE Peer: 192.144.80.90</t>
+  </si>
+  <si>
+    <t>8   IKE Peer: 182.163.98.81</t>
+  </si>
+  <si>
+    <t>9   IKE Peer: 202.84.44.65</t>
+  </si>
+  <si>
+    <t>Session-id:45244, Status:UP-ACTIVE, IKE count:1, CHILD count:1</t>
+  </si>
+  <si>
+    <t>3465321743 103.17.181.122/4500                                 20.224.142.31/4500                                       READY    RESPONDER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Life/Active Time: 86400/784 sec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          ESP spi in/out: 0x98dca5af/0xc881f19d  </t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -4475,7 +4475,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -4538,7 +4538,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>155</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -4580,7 +4580,7 @@
         <v>96</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -4594,7 +4594,7 @@
         <v>96</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -4622,7 +4622,7 @@
         <v>96</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -4664,7 +4664,7 @@
         <v>8</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>209</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -4790,7 +4790,7 @@
         <v>96</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>161</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23" spans="5:5" x14ac:dyDescent="0.25">
@@ -4805,121 +4805,106 @@
     </row>
     <row r="25" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E25" s="11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="26" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E26" s="11" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E27" s="11" t="s">
-        <v>112</v>
+        <v>165</v>
       </c>
     </row>
     <row r="28" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E28" s="11" t="s">
-        <v>163</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E29" s="11" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E30" s="11" t="s">
-        <v>165</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E31" s="11" t="s">
-        <v>213</v>
+      <c r="E31" s="9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E32" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="33" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E33" s="11" t="s">
-        <v>136</v>
+      <c r="E33" s="9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E34" s="9" t="s">
-        <v>8</v>
+      <c r="E34" s="11" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="35" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E35" s="11" t="s">
-        <v>137</v>
+      <c r="E35" s="9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="36" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E36" s="9" t="s">
-        <v>8</v>
+      <c r="E36" s="11" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="37" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E37" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="38" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E38" s="9" t="s">
-        <v>8</v>
+      <c r="E38" s="11" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="39" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E39" s="11" t="s">
-        <v>139</v>
+        <v>216</v>
       </c>
     </row>
     <row r="40" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E40" s="11" t="s">
-        <v>215</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E41" s="11" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="42" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E42" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="43" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E43" s="11" t="s">
-        <v>143</v>
+        <v>218</v>
       </c>
     </row>
     <row r="44" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E44" s="11" t="s">
-        <v>144</v>
+      <c r="E44" s="9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="45" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E45" s="11" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="46" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E46" s="11" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="47" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E47" s="9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="48" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E48" s="11" t="s">
         <v>55</v>
       </c>
     </row>

</xml_diff>